<commit_message>
docs: adicionar Gemma 4 e MiniMax ao comparativo de modelos
MiniMax (M1/M2): escala datacenter (229-456B), minimo 64GB -> impossivel local.
Gemma 4 (Apache-2.0, function calling): E4B e rival do Qwen3-4B, mas PLE infla
memoria (Q8 nao cabe nos 8GB) + template/tools diferentes + arquitetura nova.
Qwen3-4B vence por fit-Q8 + drop-in + maturidade. 27 modelos no total.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/comparativo_modelos_LLM.xlsx
+++ b/docs/comparativo_modelos_LLM.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Fontes e Metodologia" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comparacao'!$A$3:$T$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comparacao'!$A$3:$T$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -125,7 +125,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -167,6 +167,11 @@
         <fgColor rgb="00006100"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007F6000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -194,7 +199,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -264,6 +269,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -646,7 +654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T23"/>
+  <dimension ref="A1:T30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -897,28 +905,28 @@
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Qwen3-30B-A3B-Instruct-2507</t>
+          <t>MiniMax-M1</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Qwen</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>MoE (3B ativos)</t>
+          <t>Hibrido MoE (lightning attn)</t>
         </is>
       </c>
       <c r="D5" s="10" t="n">
-        <v>30</v>
+        <v>456</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>3</v>
+        <v>45.9</v>
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>262K</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="G5" s="11" t="inlineStr">
@@ -927,7 +935,7 @@
         </is>
       </c>
       <c r="H5" s="10" t="n">
-        <v>18</v>
+        <v>250</v>
       </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
@@ -936,86 +944,94 @@
       </c>
       <c r="J5" s="11" t="inlineStr">
         <is>
-          <t>~0 livre</t>
+          <t>~0 (impossivel)</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>~5-9</t>
-        </is>
-      </c>
-      <c r="L5" s="10" t="n">
-        <v>69.09999999999999</v>
-      </c>
-      <c r="M5" s="10" t="n">
-        <v>54.8</v>
-      </c>
-      <c r="N5" s="10" t="n">
-        <v>83.7</v>
-      </c>
-      <c r="O5" s="10" t="n">
-        <v>58.6</v>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="M5" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="N5" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="O5" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
       </c>
       <c r="P5" s="10" t="inlineStr">
         <is>
-          <t>Bom (119 idiomas)</t>
+          <t>Bom (multiling.)</t>
         </is>
       </c>
       <c r="Q5" s="10" t="inlineStr">
         <is>
-          <t>Nativo (forte)</t>
+          <t>Nativo (agentic)</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Muito Alto</t>
         </is>
       </c>
       <c r="S5" s="13" t="inlineStr">
         <is>
-          <t>Mesmo problema de memoria do 35B; o 4B-2507 empata com ele</t>
+          <t>Escala datacenter (456B totais): impossivel local; so servidor/API</t>
         </is>
       </c>
       <c r="T5" s="11" t="inlineStr">
         <is>
-          <t>HF Qwen3-4B-2507 card</t>
+          <t>arXiv 2506.13585</t>
         </is>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>Gemma 3 27B</t>
+          <t>MiniMax-M2</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>Densa</t>
+          <t>MoE (10B ativos)</t>
         </is>
       </c>
       <c r="D6" s="15" t="n">
-        <v>27</v>
+        <v>229</v>
       </c>
       <c r="E6" s="15" t="n">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>128K</t>
+          <t>196K</t>
         </is>
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>Gemma (restritiva)</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="H6" s="15" t="n">
-        <v>16</v>
+        <v>130</v>
       </c>
       <c r="I6" s="12" t="inlineStr">
         <is>
@@ -1024,22 +1040,22 @@
       </c>
       <c r="J6" s="16" t="inlineStr">
         <is>
-          <t>~0 livre</t>
+          <t>~0 (impossivel)</t>
         </is>
       </c>
       <c r="K6" s="15" t="inlineStr">
         <is>
-          <t>~2-4</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
         <is>
-          <t>n/d (52.2 CoT)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="M6" s="15" t="inlineStr">
         <is>
-          <t>24.3</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="N6" s="15" t="inlineStr">
@@ -1054,27 +1070,27 @@
       </c>
       <c r="P6" s="15" t="inlineStr">
         <is>
-          <t>Excelente (140 idiomas)</t>
+          <t>Bom (multiling.)</t>
         </is>
       </c>
       <c r="Q6" s="15" t="inlineStr">
         <is>
-          <t>Suportado</t>
+          <t>Nativo (agentic forte)</t>
         </is>
       </c>
       <c r="R6" s="15" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Muito Alto</t>
         </is>
       </c>
       <c r="S6" s="17" t="inlineStr">
         <is>
-          <t>Otimo multilingue, mas pesado demais p/ este hardware</t>
+          <t>229B totais: minimo ~64GB (IQ1_S). Impossivel neste hardware; servidor/API</t>
         </is>
       </c>
       <c r="T6" s="16" t="inlineStr">
         <is>
-          <t>HF google/gemma-3</t>
+          <t>HF unsloth/MiniMax-M2-GGUF</t>
         </is>
       </c>
     </row>
@@ -1177,12 +1193,12 @@
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Phi-4 (14B)</t>
+          <t>Gemma 4 31B Dense</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
@@ -1191,37 +1207,37 @@
         </is>
       </c>
       <c r="D8" s="15" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="E8" s="15" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>16K</t>
+          <t>256K</t>
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>Apache-2.0</t>
         </is>
       </c>
       <c r="H8" s="15" t="n">
-        <v>9</v>
-      </c>
-      <c r="I8" s="18" t="inlineStr">
-        <is>
-          <t>Parcial</t>
+        <v>19</v>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>Nao</t>
         </is>
       </c>
       <c r="J8" s="16" t="inlineStr">
         <is>
-          <t>~6-7 GB</t>
+          <t>~0 livre</t>
         </is>
       </c>
       <c r="K8" s="15" t="inlineStr">
         <is>
-          <t>~8-12</t>
+          <t>~2-3</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
@@ -1241,39 +1257,39 @@
       </c>
       <c r="O8" s="15" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>n/d (t2-bench 86.4)</t>
         </is>
       </c>
       <c r="P8" s="15" t="inlineStr">
         <is>
-          <t>Razoavel (EN-centrico)</t>
+          <t>Excelente (140 idiomas)</t>
         </is>
       </c>
       <c r="Q8" s="15" t="inlineStr">
         <is>
-          <t>Suportado</t>
+          <t>Nativo (FC)</t>
         </is>
       </c>
       <c r="R8" s="15" t="inlineStr">
         <is>
-          <t>Alto (STEM)</t>
+          <t>Muito Alto</t>
         </is>
       </c>
       <c r="S8" s="17" t="inlineStr">
         <is>
-          <t>Forte em raciocinio/STEM; contexto curto (16K) e offload parcial</t>
+          <t>Top de qualidade aberta (AIME 89.2), mas 31B denso pesa demais aqui</t>
         </is>
       </c>
       <c r="T8" s="16" t="inlineStr">
         <is>
-          <t>HF microsoft/phi-4</t>
+          <t>blog.google/gemma-4</t>
         </is>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Qwen3-14B</t>
+          <t>Qwen3-30B-A3B-Instruct-2507</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
@@ -1283,18 +1299,18 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Densa</t>
+          <t>MoE (3B ativos)</t>
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>128K</t>
+          <t>262K</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
@@ -1303,46 +1319,38 @@
         </is>
       </c>
       <c r="H9" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="I9" s="18" t="inlineStr">
-        <is>
-          <t>Parcial</t>
+        <v>18</v>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>Nao</t>
         </is>
       </c>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>~6-7 GB</t>
+          <t>~0 livre</t>
         </is>
       </c>
       <c r="K9" s="10" t="inlineStr">
         <is>
-          <t>~8-12</t>
-        </is>
-      </c>
-      <c r="L9" s="10" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="M9" s="10" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="N9" s="10" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="O9" s="10" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
+          <t>~5-9</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="n">
+        <v>69.09999999999999</v>
+      </c>
+      <c r="M9" s="10" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="N9" s="10" t="n">
+        <v>83.7</v>
+      </c>
+      <c r="O9" s="10" t="n">
+        <v>58.6</v>
       </c>
       <c r="P9" s="10" t="inlineStr">
         <is>
-          <t>Bom</t>
+          <t>Bom (119 idiomas)</t>
         </is>
       </c>
       <c r="Q9" s="10" t="inlineStr">
@@ -1357,19 +1365,19 @@
       </c>
       <c r="S9" s="13" t="inlineStr">
         <is>
-          <t>Bom equilibrio qualidade, mas nao cabe 100% na VRAM (offload parcial)</t>
+          <t>Mesmo problema de memoria do 35B; o 4B-2507 empata com ele</t>
         </is>
       </c>
       <c r="T9" s="11" t="inlineStr">
         <is>
-          <t>HF Qwen3 / insiderllm</t>
+          <t>HF Qwen3-4B-2507 card</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>Gemma 3 12B</t>
+          <t>Gemma 3 27B</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
@@ -1383,10 +1391,10 @@
         </is>
       </c>
       <c r="D10" s="15" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
@@ -1399,31 +1407,31 @@
         </is>
       </c>
       <c r="H10" s="15" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="I10" s="18" t="inlineStr">
-        <is>
-          <t>Parcial</t>
+        <v>16</v>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>Nao</t>
         </is>
       </c>
       <c r="J10" s="16" t="inlineStr">
         <is>
-          <t>~7-8 GB</t>
+          <t>~0 livre</t>
         </is>
       </c>
       <c r="K10" s="15" t="inlineStr">
         <is>
-          <t>~12-18</t>
+          <t>~2-4</t>
         </is>
       </c>
       <c r="L10" s="15" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>n/d (52.2 CoT)</t>
         </is>
       </c>
       <c r="M10" s="15" t="inlineStr">
         <is>
-          <t>25.4</t>
+          <t>24.3</t>
         </is>
       </c>
       <c r="N10" s="15" t="inlineStr">
@@ -1448,12 +1456,12 @@
       </c>
       <c r="R10" s="15" t="inlineStr">
         <is>
-          <t>Medio-Alto</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="S10" s="17" t="inlineStr">
         <is>
-          <t>Multilingue forte; cabe quase 100% em VRAM com contexto modesto</t>
+          <t>Otimo multilingue, mas pesado demais p/ este hardware</t>
         </is>
       </c>
       <c r="T10" s="16" t="inlineStr">
@@ -1465,28 +1473,28 @@
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Mistral Small 3 (24B)</t>
+          <t>Gemma 4 26B-A4B (MoE)</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Mistral</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Densa</t>
+          <t>MoE (3.8B ativos)</t>
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>24</v>
+        <v>3.8</v>
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>32K</t>
+          <t>256K</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -1495,7 +1503,7 @@
         </is>
       </c>
       <c r="H11" s="10" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
@@ -1534,12 +1542,12 @@
       </c>
       <c r="P11" s="10" t="inlineStr">
         <is>
-          <t>Bom (idiomas EU + PT)</t>
+          <t>Excelente (140 idiomas)</t>
         </is>
       </c>
       <c r="Q11" s="10" t="inlineStr">
         <is>
-          <t>Nativo</t>
+          <t>Nativo (FC)</t>
         </is>
       </c>
       <c r="R11" s="10" t="inlineStr">
@@ -1549,24 +1557,24 @@
       </c>
       <c r="S11" s="13" t="inlineStr">
         <is>
-          <t>Forte, mas 24B pesa demais aqui</t>
+          <t>MoE forte (AIME 88.3), mas 26B totais nao cabem (mesmo trap do 35B)</t>
         </is>
       </c>
       <c r="T11" s="11" t="inlineStr">
         <is>
-          <t>Mistral AI</t>
+          <t>blog.google/gemma-4</t>
         </is>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Granite 3.3 8B</t>
+          <t>Mistral Small 3 (24B)</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>Mistral</t>
         </is>
       </c>
       <c r="C12" s="16" t="inlineStr">
@@ -1575,14 +1583,14 @@
         </is>
       </c>
       <c r="D12" s="15" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>128K</t>
+          <t>32K</t>
         </is>
       </c>
       <c r="G12" s="16" t="inlineStr">
@@ -1591,21 +1599,21 @@
         </is>
       </c>
       <c r="H12" s="15" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="I12" s="19" t="inlineStr">
-        <is>
-          <t>Sim</t>
+        <v>14</v>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>Nao</t>
         </is>
       </c>
       <c r="J12" s="16" t="inlineStr">
         <is>
-          <t>~9-10 GB</t>
+          <t>~0-2 GB</t>
         </is>
       </c>
       <c r="K12" s="15" t="inlineStr">
         <is>
-          <t>~18-28</t>
+          <t>~3-5</t>
         </is>
       </c>
       <c r="L12" s="15" t="inlineStr">
@@ -1630,39 +1638,39 @@
       </c>
       <c r="P12" s="15" t="inlineStr">
         <is>
-          <t>Razoavel (12 idiomas)</t>
+          <t>Bom (idiomas EU + PT)</t>
         </is>
       </c>
       <c r="Q12" s="15" t="inlineStr">
         <is>
-          <t>Nativo (projetado p/ tools)</t>
+          <t>Nativo</t>
         </is>
       </c>
       <c r="R12" s="15" t="inlineStr">
         <is>
-          <t>Medio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="S12" s="17" t="inlineStr">
         <is>
-          <t>Cabe 100% na VRAM; bom p/ tool calling empresarial</t>
+          <t>Forte, mas 24B pesa demais aqui</t>
         </is>
       </c>
       <c r="T12" s="16" t="inlineStr">
         <is>
-          <t>IBM Granite</t>
+          <t>Mistral AI</t>
         </is>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>Llama 3.1 8B Instruct</t>
+          <t>Phi-4 (14B)</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
@@ -1671,37 +1679,37 @@
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>128K</t>
+          <t>16K</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>Llama 3.1 (custom)</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="H13" s="10" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="I13" s="19" t="inlineStr">
-        <is>
-          <t>Sim</t>
+        <v>9</v>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
+        <is>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="J13" s="11" t="inlineStr">
         <is>
-          <t>~9-10 GB</t>
+          <t>~6-7 GB</t>
         </is>
       </c>
       <c r="K13" s="10" t="inlineStr">
         <is>
-          <t>~18-28</t>
+          <t>~8-12</t>
         </is>
       </c>
       <c r="L13" s="10" t="inlineStr">
@@ -1711,49 +1719,49 @@
       </c>
       <c r="M13" s="10" t="inlineStr">
         <is>
-          <t>32.8</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="N13" s="10" t="inlineStr">
         <is>
-          <t>80.4</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="O13" s="10" t="inlineStr">
         <is>
-          <t>76.1</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="P13" s="10" t="inlineStr">
         <is>
-          <t>Bom (8 idiomas, inc. PT)</t>
+          <t>Razoavel (EN-centrico)</t>
         </is>
       </c>
       <c r="Q13" s="10" t="inlineStr">
         <is>
-          <t>Nativo (BFCL 76)</t>
+          <t>Suportado</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
         <is>
-          <t>Medio</t>
+          <t>Alto (STEM)</t>
         </is>
       </c>
       <c r="S13" s="13" t="inlineStr">
         <is>
-          <t>Cabe 100% na VRAM; tool calling forte; PT-BR oficial</t>
+          <t>Forte em raciocinio/STEM; contexto curto (16K) e offload parcial</t>
         </is>
       </c>
       <c r="T13" s="11" t="inlineStr">
         <is>
-          <t>HF meta-llama / Llama3 paper</t>
+          <t>HF microsoft/phi-4</t>
         </is>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Qwen3-8B</t>
+          <t>Qwen3-14B</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
@@ -1767,10 +1775,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
@@ -1783,21 +1791,21 @@
         </is>
       </c>
       <c r="H14" s="15" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="I14" s="19" t="inlineStr">
-        <is>
-          <t>Sim</t>
+        <v>9</v>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="J14" s="16" t="inlineStr">
         <is>
-          <t>~9-10 GB</t>
+          <t>~6-7 GB</t>
         </is>
       </c>
       <c r="K14" s="15" t="inlineStr">
         <is>
-          <t>~18-28</t>
+          <t>~8-12</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
@@ -1822,7 +1830,7 @@
       </c>
       <c r="P14" s="15" t="inlineStr">
         <is>
-          <t>Bom (119 idiomas)</t>
+          <t>Bom</t>
         </is>
       </c>
       <c r="Q14" s="15" t="inlineStr">
@@ -1832,12 +1840,12 @@
       </c>
       <c r="R14" s="15" t="inlineStr">
         <is>
-          <t>Medio-Alto</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="S14" s="17" t="inlineStr">
         <is>
-          <t>DROP-IN no codigo atual; cabe 100% na VRAM; ja foi usado no projeto</t>
+          <t>Bom equilibrio qualidade, mas nao cabe 100% na VRAM (offload parcial)</t>
         </is>
       </c>
       <c r="T14" s="16" t="inlineStr">
@@ -1849,12 +1857,12 @@
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Ministral 8B (Ministral 3)</t>
+          <t>Gemma 3 12B</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Mistral</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
@@ -1863,10 +1871,10 @@
         </is>
       </c>
       <c r="D15" s="10" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
@@ -1875,25 +1883,25 @@
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>Mistral Research/Comm.</t>
+          <t>Gemma (restritiva)</t>
         </is>
       </c>
       <c r="H15" s="10" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="I15" s="19" t="inlineStr">
-        <is>
-          <t>Sim</t>
+        <v>7.3</v>
+      </c>
+      <c r="I15" s="18" t="inlineStr">
+        <is>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="J15" s="11" t="inlineStr">
         <is>
-          <t>~9-10 GB</t>
+          <t>~7-8 GB</t>
         </is>
       </c>
       <c r="K15" s="10" t="inlineStr">
         <is>
-          <t>~18-28</t>
+          <t>~12-18</t>
         </is>
       </c>
       <c r="L15" s="10" t="inlineStr">
@@ -1903,7 +1911,7 @@
       </c>
       <c r="M15" s="10" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>25.4</t>
         </is>
       </c>
       <c r="N15" s="10" t="inlineStr">
@@ -1918,34 +1926,34 @@
       </c>
       <c r="P15" s="10" t="inlineStr">
         <is>
-          <t>Bom (idiomas EU + PT)</t>
+          <t>Excelente (140 idiomas)</t>
         </is>
       </c>
       <c r="Q15" s="10" t="inlineStr">
         <is>
-          <t>Nativo</t>
+          <t>Suportado</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
         <is>
-          <t>Medio</t>
+          <t>Medio-Alto</t>
         </is>
       </c>
       <c r="S15" s="13" t="inlineStr">
         <is>
-          <t>Cabe 100% na VRAM; eficiente; supera Gemma 12B em parte dos evals</t>
+          <t>Multilingue forte; cabe quase 100% em VRAM com contexto modesto</t>
         </is>
       </c>
       <c r="T15" s="11" t="inlineStr">
         <is>
-          <t>Ministral 3 paper (arXiv)</t>
+          <t>HF google/gemma-3</t>
         </is>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>Gemma 3 4B</t>
+          <t>Gemma 4 12B</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
@@ -1955,186 +1963,194 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
+          <t>Densa (multimodal)</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>128K</t>
+        </is>
+      </c>
+      <c r="G16" s="16" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>~7-8 GB</t>
+        </is>
+      </c>
+      <c r="K16" s="15" t="inlineStr">
+        <is>
+          <t>~12-18</t>
+        </is>
+      </c>
+      <c r="L16" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="M16" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="N16" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="O16" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="P16" s="15" t="inlineStr">
+        <is>
+          <t>Excelente (140 idiomas)</t>
+        </is>
+      </c>
+      <c r="Q16" s="15" t="inlineStr">
+        <is>
+          <t>Nativo (FC)</t>
+        </is>
+      </c>
+      <c r="R16" s="15" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="S16" s="17" t="inlineStr">
+        <is>
+          <t>Multimodal forte; cabe quase 100% com ctx modesto; FC nativo</t>
+        </is>
+      </c>
+      <c r="T16" s="16" t="inlineStr">
+        <is>
+          <t>ai.google.dev/gemma</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Granite 3.3 8B</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
           <t>Densa</t>
         </is>
       </c>
-      <c r="D16" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="E16" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="F16" s="16" t="inlineStr">
+      <c r="D17" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
         <is>
           <t>128K</t>
         </is>
       </c>
-      <c r="G16" s="16" t="inlineStr">
-        <is>
-          <t>Gemma (restritiva)</t>
-        </is>
-      </c>
-      <c r="H16" s="15" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="I16" s="19" t="inlineStr">
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I17" s="19" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="J16" s="16" t="inlineStr">
-        <is>
-          <t>~10-11 GB</t>
-        </is>
-      </c>
-      <c r="K16" s="15" t="inlineStr">
-        <is>
-          <t>~30-45</t>
-        </is>
-      </c>
-      <c r="L16" s="15" t="inlineStr">
-        <is>
-          <t>n/d (Glob-MMLU 57)</t>
-        </is>
-      </c>
-      <c r="M16" s="15" t="inlineStr">
-        <is>
-          <t>15.0</t>
-        </is>
-      </c>
-      <c r="N16" s="15" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="O16" s="15" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="P16" s="15" t="inlineStr">
-        <is>
-          <t>Excelente (140 idiomas)</t>
-        </is>
-      </c>
-      <c r="Q16" s="15" t="inlineStr">
-        <is>
-          <t>Suportado</t>
-        </is>
-      </c>
-      <c r="R16" s="15" t="inlineStr">
+      <c r="J17" s="11" t="inlineStr">
+        <is>
+          <t>~9-10 GB</t>
+        </is>
+      </c>
+      <c r="K17" s="10" t="inlineStr">
+        <is>
+          <t>~18-28</t>
+        </is>
+      </c>
+      <c r="L17" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="M17" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="N17" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="O17" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="P17" s="10" t="inlineStr">
+        <is>
+          <t>Razoavel (12 idiomas)</t>
+        </is>
+      </c>
+      <c r="Q17" s="10" t="inlineStr">
+        <is>
+          <t>Nativo (projetado p/ tools)</t>
+        </is>
+      </c>
+      <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="S16" s="17" t="inlineStr">
-        <is>
-          <t>MELHOR multilingue leve; cabe folgado; tool calling menos maduro</t>
-        </is>
-      </c>
-      <c r="T16" s="16" t="inlineStr">
-        <is>
-          <t>HF google/gemma-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="20" t="inlineStr">
-        <is>
-          <t>Qwen3-4B-Instruct-2507  *</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Qwen</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>Densa</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E17" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="F17" s="11" t="inlineStr">
-        <is>
-          <t>262K</t>
-        </is>
-      </c>
-      <c r="G17" s="11" t="inlineStr">
-        <is>
-          <t>Apache-2.0</t>
-        </is>
-      </c>
-      <c r="H17" s="10" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="I17" s="19" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="J17" s="11" t="inlineStr">
-        <is>
-          <t>~10-11 GB livre</t>
-        </is>
-      </c>
-      <c r="K17" s="10" t="inlineStr">
-        <is>
-          <t>~30-45</t>
-        </is>
-      </c>
-      <c r="L17" s="10" t="n">
-        <v>69.59999999999999</v>
-      </c>
-      <c r="M17" s="10" t="n">
-        <v>62</v>
-      </c>
-      <c r="N17" s="10" t="n">
-        <v>83.40000000000001</v>
-      </c>
-      <c r="O17" s="10" t="n">
-        <v>61.9</v>
-      </c>
-      <c r="P17" s="10" t="inlineStr">
-        <is>
-          <t>Bom (119 idiomas)</t>
-        </is>
-      </c>
-      <c r="Q17" s="10" t="inlineStr">
-        <is>
-          <t>Nativo (BFCL 61.9)</t>
-        </is>
-      </c>
-      <c r="R17" s="10" t="inlineStr">
-        <is>
-          <t>Medio-Alto</t>
-        </is>
-      </c>
-      <c r="S17" s="20" t="inlineStr">
-        <is>
-          <t>ESCOLHA TOP: empata/supera o 30B-A3B; DROP-IN; ja baixado; deixa a maquina livre</t>
+      <c r="S17" s="13" t="inlineStr">
+        <is>
+          <t>Cabe 100% na VRAM; bom p/ tool calling empresarial</t>
         </is>
       </c>
       <c r="T17" s="11" t="inlineStr">
         <is>
-          <t>HF Qwen/Qwen3-4B-Instruct-2507</t>
+          <t>IBM Granite</t>
         </is>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>Phi-4-mini (3.8B)</t>
+          <t>Llama 3.1 8B Instruct</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="C18" s="16" t="inlineStr">
@@ -2143,10 +2159,10 @@
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>3.8</v>
+        <v>8</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>3.8</v>
+        <v>8</v>
       </c>
       <c r="F18" s="16" t="inlineStr">
         <is>
@@ -2155,11 +2171,11 @@
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>Llama 3.1 (custom)</t>
         </is>
       </c>
       <c r="H18" s="15" t="n">
-        <v>2.5</v>
+        <v>4.9</v>
       </c>
       <c r="I18" s="19" t="inlineStr">
         <is>
@@ -2168,38 +2184,42 @@
       </c>
       <c r="J18" s="16" t="inlineStr">
         <is>
-          <t>~10-11 GB</t>
+          <t>~9-10 GB</t>
         </is>
       </c>
       <c r="K18" s="15" t="inlineStr">
         <is>
-          <t>~30-45</t>
-        </is>
-      </c>
-      <c r="L18" s="15" t="n">
-        <v>52.8</v>
-      </c>
-      <c r="M18" s="15" t="n">
-        <v>25.2</v>
+          <t>~18-28</t>
+        </is>
+      </c>
+      <c r="L18" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="M18" s="15" t="inlineStr">
+        <is>
+          <t>32.8</t>
+        </is>
       </c>
       <c r="N18" s="15" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>80.4</t>
         </is>
       </c>
       <c r="O18" s="15" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>76.1</t>
         </is>
       </c>
       <c r="P18" s="15" t="inlineStr">
         <is>
-          <t>Razoavel</t>
+          <t>Bom (8 idiomas, inc. PT)</t>
         </is>
       </c>
       <c r="Q18" s="15" t="inlineStr">
         <is>
-          <t>Suportado</t>
+          <t>Nativo (BFCL 76)</t>
         </is>
       </c>
       <c r="R18" s="15" t="inlineStr">
@@ -2209,24 +2229,24 @@
       </c>
       <c r="S18" s="17" t="inlineStr">
         <is>
-          <t>Forte em mat/STEM p/ o tamanho; PT-BR mediano</t>
+          <t>Cabe 100% na VRAM; tool calling forte; PT-BR oficial</t>
         </is>
       </c>
       <c r="T18" s="16" t="inlineStr">
         <is>
-          <t>HF microsoft/Phi-4-mini-instruct</t>
+          <t>HF meta-llama / Llama3 paper</t>
         </is>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Llama 3.2 3B Instruct</t>
+          <t>Qwen3-8B</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>Qwen</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
@@ -2235,10 +2255,10 @@
         </is>
       </c>
       <c r="D19" s="10" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E19" s="10" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
@@ -2247,11 +2267,11 @@
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>Llama 3.2 (custom)</t>
+          <t>Apache-2.0</t>
         </is>
       </c>
       <c r="H19" s="10" t="n">
-        <v>2</v>
+        <v>4.9</v>
       </c>
       <c r="I19" s="19" t="inlineStr">
         <is>
@@ -2260,61 +2280,69 @@
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>~11-12 GB</t>
+          <t>~9-10 GB</t>
         </is>
       </c>
       <c r="K19" s="10" t="inlineStr">
         <is>
-          <t>~35-50</t>
-        </is>
-      </c>
-      <c r="L19" s="10" t="n">
-        <v>39.2</v>
-      </c>
-      <c r="M19" s="10" t="n">
-        <v>32.8</v>
-      </c>
-      <c r="N19" s="10" t="n">
-        <v>77.40000000000001</v>
-      </c>
-      <c r="O19" s="10" t="n">
-        <v>67</v>
+          <t>~18-28</t>
+        </is>
+      </c>
+      <c r="L19" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="M19" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="N19" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="O19" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
       </c>
       <c r="P19" s="10" t="inlineStr">
         <is>
-          <t>Bom (8 idiomas, inc. PT)</t>
+          <t>Bom (119 idiomas)</t>
         </is>
       </c>
       <c r="Q19" s="10" t="inlineStr">
         <is>
-          <t>Nativo (BFCL 67)</t>
+          <t>Nativo (forte)</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
         <is>
-          <t>Medio-Basico</t>
+          <t>Medio-Alto</t>
         </is>
       </c>
       <c r="S19" s="13" t="inlineStr">
         <is>
-          <t>Leve, tool calling decente; conhecimento limitado (MMLU-Pro 39)</t>
+          <t>DROP-IN no codigo atual; cabe 100% na VRAM; ja foi usado no projeto</t>
         </is>
       </c>
       <c r="T19" s="11" t="inlineStr">
         <is>
-          <t>HF meta-llama/Llama-3.2-3B</t>
+          <t>HF Qwen3 / insiderllm</t>
         </is>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>Qwen3-1.7B</t>
+          <t>Ministral 8B (Ministral 3)</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>Qwen</t>
+          <t>Mistral</t>
         </is>
       </c>
       <c r="C20" s="16" t="inlineStr">
@@ -2323,23 +2351,23 @@
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>1.7</v>
+        <v>8</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>1.7</v>
+        <v>8</v>
       </c>
       <c r="F20" s="16" t="inlineStr">
         <is>
-          <t>32K</t>
+          <t>128K</t>
         </is>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>Apache-2.0</t>
+          <t>Mistral Research/Comm.</t>
         </is>
       </c>
       <c r="H20" s="15" t="n">
-        <v>1.1</v>
+        <v>4.9</v>
       </c>
       <c r="I20" s="19" t="inlineStr">
         <is>
@@ -2348,12 +2376,12 @@
       </c>
       <c r="J20" s="16" t="inlineStr">
         <is>
-          <t>~12-13 GB</t>
+          <t>~9-10 GB</t>
         </is>
       </c>
       <c r="K20" s="15" t="inlineStr">
         <is>
-          <t>~50-70</t>
+          <t>~18-28</t>
         </is>
       </c>
       <c r="L20" s="15" t="inlineStr">
@@ -2378,7 +2406,7 @@
       </c>
       <c r="P20" s="15" t="inlineStr">
         <is>
-          <t>Razoavel</t>
+          <t>Bom (idiomas EU + PT)</t>
         </is>
       </c>
       <c r="Q20" s="15" t="inlineStr">
@@ -2388,45 +2416,45 @@
       </c>
       <c r="R20" s="15" t="inlineStr">
         <is>
-          <t>Basico+</t>
+          <t>Medio</t>
         </is>
       </c>
       <c r="S20" s="17" t="inlineStr">
         <is>
-          <t>Muito rapido; DROP-IN; qualidade limitada p/ tarefas complexas</t>
+          <t>Cabe 100% na VRAM; eficiente; supera Gemma 12B em parte dos evals</t>
         </is>
       </c>
       <c r="T20" s="16" t="inlineStr">
         <is>
-          <t>HF Qwen3</t>
+          <t>Ministral 3 paper (arXiv)</t>
         </is>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>SmolLM2 1.7B</t>
+          <t>Gemma 4 E4B</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>HuggingFace</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>Densa</t>
+          <t>Densa PLE (multimodal)</t>
         </is>
       </c>
       <c r="D21" s="10" t="n">
-        <v>1.7</v>
+        <v>4.5</v>
       </c>
       <c r="E21" s="10" t="n">
-        <v>1.7</v>
+        <v>4.5</v>
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>8K</t>
+          <t>128K</t>
         </is>
       </c>
       <c r="G21" s="11" t="inlineStr">
@@ -2435,21 +2463,21 @@
         </is>
       </c>
       <c r="H21" s="10" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="I21" s="19" t="inlineStr">
-        <is>
-          <t>Sim</t>
+        <v>5</v>
+      </c>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>Q4 so</t>
         </is>
       </c>
       <c r="J21" s="11" t="inlineStr">
         <is>
-          <t>~12-13 GB</t>
+          <t>~10-11 GB</t>
         </is>
       </c>
       <c r="K21" s="10" t="inlineStr">
         <is>
-          <t>~50-70</t>
+          <t>~25-40</t>
         </is>
       </c>
       <c r="L21" s="10" t="inlineStr">
@@ -2474,218 +2502,870 @@
       </c>
       <c r="P21" s="10" t="inlineStr">
         <is>
-          <t>Fraco (EN-centrico)</t>
+          <t>Excelente (140 idiomas)</t>
         </is>
       </c>
       <c r="Q21" s="10" t="inlineStr">
         <is>
-          <t>Limitado</t>
+          <t>Nativo (FC)</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
-          <t>Basico</t>
+          <t>Medio-Alto</t>
         </is>
       </c>
       <c r="S21" s="13" t="inlineStr">
         <is>
-          <t>Leve, mas fraco em PT-BR e tools</t>
+          <t>Rival direto do Qwen3-4B; PLE infla memoria (Q8 ~9-10GB nao cabe -&gt; roda Q4); template/FC diferentes</t>
         </is>
       </c>
       <c r="T21" s="11" t="inlineStr">
         <is>
-          <t>HF HuggingFaceTB/SmolLM2</t>
+          <t>ai.google.dev/gemma</t>
         </is>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
+          <t>Gemma 3 4B</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>Densa</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E22" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <t>128K</t>
+        </is>
+      </c>
+      <c r="G22" s="16" t="inlineStr">
+        <is>
+          <t>Gemma (restritiva)</t>
+        </is>
+      </c>
+      <c r="H22" s="15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I22" s="19" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J22" s="16" t="inlineStr">
+        <is>
+          <t>~10-11 GB</t>
+        </is>
+      </c>
+      <c r="K22" s="15" t="inlineStr">
+        <is>
+          <t>~30-45</t>
+        </is>
+      </c>
+      <c r="L22" s="15" t="inlineStr">
+        <is>
+          <t>n/d (Glob-MMLU 57)</t>
+        </is>
+      </c>
+      <c r="M22" s="15" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="N22" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="O22" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="P22" s="15" t="inlineStr">
+        <is>
+          <t>Excelente (140 idiomas)</t>
+        </is>
+      </c>
+      <c r="Q22" s="15" t="inlineStr">
+        <is>
+          <t>Suportado</t>
+        </is>
+      </c>
+      <c r="R22" s="15" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="S22" s="17" t="inlineStr">
+        <is>
+          <t>MELHOR multilingue leve; cabe folgado; tool calling menos maduro</t>
+        </is>
+      </c>
+      <c r="T22" s="16" t="inlineStr">
+        <is>
+          <t>HF google/gemma-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="42" customHeight="1">
+      <c r="A23" s="20" t="inlineStr">
+        <is>
+          <t>Qwen3-4B-Instruct-2507  *</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Densa</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>262K</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I23" s="19" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J23" s="11" t="inlineStr">
+        <is>
+          <t>~10-11 GB livre</t>
+        </is>
+      </c>
+      <c r="K23" s="10" t="inlineStr">
+        <is>
+          <t>~30-45</t>
+        </is>
+      </c>
+      <c r="L23" s="10" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="M23" s="10" t="n">
+        <v>62</v>
+      </c>
+      <c r="N23" s="10" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="O23" s="10" t="n">
+        <v>61.9</v>
+      </c>
+      <c r="P23" s="10" t="inlineStr">
+        <is>
+          <t>Bom (119 idiomas)</t>
+        </is>
+      </c>
+      <c r="Q23" s="10" t="inlineStr">
+        <is>
+          <t>Nativo (BFCL 61.9)</t>
+        </is>
+      </c>
+      <c r="R23" s="10" t="inlineStr">
+        <is>
+          <t>Medio-Alto</t>
+        </is>
+      </c>
+      <c r="S23" s="20" t="inlineStr">
+        <is>
+          <t>ESCOLHA TOP: empata/supera o 30B-A3B; DROP-IN; ja baixado; deixa a maquina livre</t>
+        </is>
+      </c>
+      <c r="T23" s="11" t="inlineStr">
+        <is>
+          <t>HF Qwen/Qwen3-4B-Instruct-2507</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="42" customHeight="1">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>Phi-4-mini (3.8B)</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Densa</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E24" s="15" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F24" s="16" t="inlineStr">
+        <is>
+          <t>128K</t>
+        </is>
+      </c>
+      <c r="G24" s="16" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="H24" s="15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I24" s="19" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J24" s="16" t="inlineStr">
+        <is>
+          <t>~10-11 GB</t>
+        </is>
+      </c>
+      <c r="K24" s="15" t="inlineStr">
+        <is>
+          <t>~30-45</t>
+        </is>
+      </c>
+      <c r="L24" s="15" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="M24" s="15" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="N24" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="O24" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="P24" s="15" t="inlineStr">
+        <is>
+          <t>Razoavel</t>
+        </is>
+      </c>
+      <c r="Q24" s="15" t="inlineStr">
+        <is>
+          <t>Suportado</t>
+        </is>
+      </c>
+      <c r="R24" s="15" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="S24" s="17" t="inlineStr">
+        <is>
+          <t>Forte em mat/STEM p/ o tamanho; PT-BR mediano</t>
+        </is>
+      </c>
+      <c r="T24" s="16" t="inlineStr">
+        <is>
+          <t>HF microsoft/Phi-4-mini-instruct</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Llama 3.2 3B Instruct</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Densa</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>128K</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>Llama 3.2 (custom)</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" s="19" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J25" s="11" t="inlineStr">
+        <is>
+          <t>~11-12 GB</t>
+        </is>
+      </c>
+      <c r="K25" s="10" t="inlineStr">
+        <is>
+          <t>~35-50</t>
+        </is>
+      </c>
+      <c r="L25" s="10" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="M25" s="10" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="N25" s="10" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="O25" s="10" t="n">
+        <v>67</v>
+      </c>
+      <c r="P25" s="10" t="inlineStr">
+        <is>
+          <t>Bom (8 idiomas, inc. PT)</t>
+        </is>
+      </c>
+      <c r="Q25" s="10" t="inlineStr">
+        <is>
+          <t>Nativo (BFCL 67)</t>
+        </is>
+      </c>
+      <c r="R25" s="10" t="inlineStr">
+        <is>
+          <t>Medio-Basico</t>
+        </is>
+      </c>
+      <c r="S25" s="13" t="inlineStr">
+        <is>
+          <t>Leve, tool calling decente; conhecimento limitado (MMLU-Pro 39)</t>
+        </is>
+      </c>
+      <c r="T25" s="11" t="inlineStr">
+        <is>
+          <t>HF meta-llama/Llama-3.2-3B</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>Gemma 4 E2B</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>Densa PLE (multimodal)</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
+        <is>
+          <t>128K</t>
+        </is>
+      </c>
+      <c r="G26" s="16" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="H26" s="15" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="I26" s="19" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J26" s="16" t="inlineStr">
+        <is>
+          <t>~11-12 GB</t>
+        </is>
+      </c>
+      <c r="K26" s="15" t="inlineStr">
+        <is>
+          <t>~40-60</t>
+        </is>
+      </c>
+      <c r="L26" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="M26" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="N26" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="O26" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="P26" s="15" t="inlineStr">
+        <is>
+          <t>Excelente (140 idiomas)</t>
+        </is>
+      </c>
+      <c r="Q26" s="15" t="inlineStr">
+        <is>
+          <t>Nativo (FC)</t>
+        </is>
+      </c>
+      <c r="R26" s="15" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="S26" s="17" t="inlineStr">
+        <is>
+          <t>Leve e multimodal; otimo multilingue; menos capaz que o E4B</t>
+        </is>
+      </c>
+      <c r="T26" s="16" t="inlineStr">
+        <is>
+          <t>ai.google.dev/gemma</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>Qwen3-1.7B</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Densa</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E27" s="10" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>32K</t>
+        </is>
+      </c>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="I27" s="19" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J27" s="11" t="inlineStr">
+        <is>
+          <t>~12-13 GB</t>
+        </is>
+      </c>
+      <c r="K27" s="10" t="inlineStr">
+        <is>
+          <t>~50-70</t>
+        </is>
+      </c>
+      <c r="L27" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="M27" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="N27" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="O27" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="P27" s="10" t="inlineStr">
+        <is>
+          <t>Razoavel</t>
+        </is>
+      </c>
+      <c r="Q27" s="10" t="inlineStr">
+        <is>
+          <t>Nativo</t>
+        </is>
+      </c>
+      <c r="R27" s="10" t="inlineStr">
+        <is>
+          <t>Basico+</t>
+        </is>
+      </c>
+      <c r="S27" s="13" t="inlineStr">
+        <is>
+          <t>Muito rapido; DROP-IN; qualidade limitada p/ tarefas complexas</t>
+        </is>
+      </c>
+      <c r="T27" s="11" t="inlineStr">
+        <is>
+          <t>HF Qwen3</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="42" customHeight="1">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>SmolLM2 1.7B</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>HuggingFace</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>Densa</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E28" s="15" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F28" s="16" t="inlineStr">
+        <is>
+          <t>8K</t>
+        </is>
+      </c>
+      <c r="G28" s="16" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="H28" s="15" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="I28" s="19" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J28" s="16" t="inlineStr">
+        <is>
+          <t>~12-13 GB</t>
+        </is>
+      </c>
+      <c r="K28" s="15" t="inlineStr">
+        <is>
+          <t>~50-70</t>
+        </is>
+      </c>
+      <c r="L28" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="M28" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="N28" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="O28" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="P28" s="15" t="inlineStr">
+        <is>
+          <t>Fraco (EN-centrico)</t>
+        </is>
+      </c>
+      <c r="Q28" s="15" t="inlineStr">
+        <is>
+          <t>Limitado</t>
+        </is>
+      </c>
+      <c r="R28" s="15" t="inlineStr">
+        <is>
+          <t>Basico</t>
+        </is>
+      </c>
+      <c r="S28" s="17" t="inlineStr">
+        <is>
+          <t>Leve, mas fraco em PT-BR e tools</t>
+        </is>
+      </c>
+      <c r="T28" s="16" t="inlineStr">
+        <is>
+          <t>HF HuggingFaceTB/SmolLM2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="42" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
           <t>Llama 3.2 1B Instruct</t>
         </is>
       </c>
-      <c r="B22" s="15" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>Meta</t>
         </is>
       </c>
-      <c r="C22" s="16" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
         <is>
           <t>Densa</t>
         </is>
       </c>
-      <c r="D22" s="15" t="n">
+      <c r="D29" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="15" t="n">
+      <c r="E29" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F22" s="16" t="inlineStr">
+      <c r="F29" s="11" t="inlineStr">
         <is>
           <t>128K</t>
         </is>
       </c>
-      <c r="G22" s="16" t="inlineStr">
+      <c r="G29" s="11" t="inlineStr">
         <is>
           <t>Llama 3.2 (custom)</t>
         </is>
       </c>
-      <c r="H22" s="15" t="n">
+      <c r="H29" s="10" t="n">
         <v>0.8</v>
       </c>
-      <c r="I22" s="19" t="inlineStr">
+      <c r="I29" s="19" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="J22" s="16" t="inlineStr">
+      <c r="J29" s="11" t="inlineStr">
         <is>
           <t>~13 GB</t>
         </is>
       </c>
-      <c r="K22" s="15" t="inlineStr">
+      <c r="K29" s="10" t="inlineStr">
         <is>
           <t>~60-90</t>
         </is>
       </c>
-      <c r="L22" s="15" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="M22" s="15" t="n">
+      <c r="L29" s="10" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="M29" s="10" t="n">
         <v>27.2</v>
       </c>
-      <c r="N22" s="15" t="n">
+      <c r="N29" s="10" t="n">
         <v>59.5</v>
       </c>
-      <c r="O22" s="15" t="n">
+      <c r="O29" s="10" t="n">
         <v>25.7</v>
       </c>
-      <c r="P22" s="15" t="inlineStr">
+      <c r="P29" s="10" t="inlineStr">
         <is>
           <t>Razoavel</t>
         </is>
       </c>
-      <c r="Q22" s="15" t="inlineStr">
+      <c r="Q29" s="10" t="inlineStr">
         <is>
           <t>Fraco (BFCL 26)</t>
         </is>
       </c>
-      <c r="R22" s="15" t="inlineStr">
+      <c r="R29" s="10" t="inlineStr">
         <is>
           <t>Basico</t>
         </is>
       </c>
-      <c r="S22" s="17" t="inlineStr">
+      <c r="S29" s="13" t="inlineStr">
         <is>
           <t>Ultra-leve; tool calling fraco; so p/ comandos simples</t>
         </is>
       </c>
-      <c r="T22" s="16" t="inlineStr">
+      <c r="T29" s="11" t="inlineStr">
         <is>
           <t>HF meta-llama/Llama-3.2-1B</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="42" customHeight="1">
-      <c r="A23" s="9" t="inlineStr">
+    <row r="30" ht="42" customHeight="1">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>Qwen3-0.6B</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>Qwen</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C30" s="16" t="inlineStr">
         <is>
           <t>Densa</t>
         </is>
       </c>
-      <c r="D23" s="10" t="n">
+      <c r="D30" s="15" t="n">
         <v>0.6</v>
       </c>
-      <c r="E23" s="10" t="n">
+      <c r="E30" s="15" t="n">
         <v>0.6</v>
       </c>
-      <c r="F23" s="11" t="inlineStr">
+      <c r="F30" s="16" t="inlineStr">
         <is>
           <t>32K</t>
         </is>
       </c>
-      <c r="G23" s="11" t="inlineStr">
+      <c r="G30" s="16" t="inlineStr">
         <is>
           <t>Apache-2.0</t>
         </is>
       </c>
-      <c r="H23" s="10" t="n">
+      <c r="H30" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="I23" s="19" t="inlineStr">
+      <c r="I30" s="19" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="J23" s="11" t="inlineStr">
+      <c r="J30" s="16" t="inlineStr">
         <is>
           <t>~13 GB</t>
         </is>
       </c>
-      <c r="K23" s="10" t="inlineStr">
+      <c r="K30" s="15" t="inlineStr">
         <is>
           <t>~80-100</t>
         </is>
       </c>
-      <c r="L23" s="10" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="M23" s="10" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="N23" s="10" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="O23" s="10" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="P23" s="10" t="inlineStr">
+      <c r="L30" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="M30" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="N30" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="O30" s="15" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="P30" s="15" t="inlineStr">
         <is>
           <t>Fraco</t>
         </is>
       </c>
-      <c r="Q23" s="10" t="inlineStr">
+      <c r="Q30" s="15" t="inlineStr">
         <is>
           <t>Nativo (limitado)</t>
         </is>
       </c>
-      <c r="R23" s="10" t="inlineStr">
+      <c r="R30" s="15" t="inlineStr">
         <is>
           <t>Basico</t>
         </is>
       </c>
-      <c r="S23" s="13" t="inlineStr">
+      <c r="S30" s="17" t="inlineStr">
         <is>
           <t>Minusculo; so p/ wake/roteamento, nao p/ conversa real</t>
         </is>
       </c>
-      <c r="T23" s="11" t="inlineStr">
+      <c r="T30" s="16" t="inlineStr">
         <is>
           <t>HF Qwen3</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:T23"/>
+  <autoFilter ref="A3:T30"/>
   <mergeCells count="2">
     <mergeCell ref="A1:T1"/>
     <mergeCell ref="A2:T2"/>
@@ -2700,7 +3380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B37"/>
+  <dimension ref="B1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2901,19 +3581,47 @@
     <row r="35" ht="24" customHeight="1">
       <c r="B35" s="25" t="inlineStr">
         <is>
+          <t>4b. Avaliados a pedido: Gemma 4 e MiniMax (jun/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="64" customHeight="1">
+      <c r="B36" s="23" t="inlineStr">
+        <is>
+          <t>MiniMax (M1/M2/M2.1): FORA por hardware, nao por qualidade. Sao modelos de escala datacenter (229B-456B totais). Mesmo com 10B ativos, os totais tem que caber na memoria: o menor GGUF do M2 (IQ1_S, 1-bit) ja sao 64 GB. No RX 580 (8GB+16GB) e fisicamente impossivel -&gt; so vLLM/SGLang em servidor ou API. E o mesmo erro do 35B, 3-13x pior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="112" customHeight="1">
+      <c r="B37" s="23" t="inlineStr">
+        <is>
+          <t>Gemma 4 (mar/2026): virou concorrente legitimo (agora Apache-2.0, function calling nativo, GGUF drop-in). O E4B e o rival direto do Qwen3-4B. Mesmo assim o Qwen vence NESTE caso por 3 motivos: (1) Q8 cabe nos 8GB de VRAM, enquanto o E4B usa Per-Layer Embeddings que inflam a memoria (Q8 ~9-10GB nao cabe -&gt; roda Q4, qualidade menor); (2) Qwen e drop-in no codigo atual (Gemma exige outro chat template e outro formato de tool calling); (3) Qwen3-4B denso e maduro no llama.cpp/Vulkan, enquanto o PLE do Gemma 4 e arquitetura nova (risco de repetir a dor bleeding-edge do 35B).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="32" customHeight="1">
+      <c r="B38" s="23" t="inlineStr">
+        <is>
+          <t>Onde o Gemma 4 PODE ganhar: PT-BR/multilingue (140 idiomas, tradicionalmente forte). Se a fluencia em portugues virar prioridade #1, vale testar o E4B aceitando Q4 + mexida no codigo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="24" customHeight="1">
+      <c r="B40" s="26" t="inlineStr">
+        <is>
           <t>5. Conclusao</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="48" customHeight="1">
-      <c r="B36" s="23" t="inlineStr">
+    <row r="41" ht="48" customHeight="1">
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t>Para um assistente de VOZ local que deve COEXISTIR com o resto da maquina, o 35B-A3B e exagero: gasta 8x mais memoria para uma qualidade que um Qwen3-4B-Instruct-2507 entrega cabendo inteiro na VRAM.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="32" customHeight="1">
-      <c r="B37" s="23" t="inlineStr">
+    <row r="42" ht="32" customHeight="1">
+      <c r="B42" s="23" t="inlineStr">
         <is>
           <t>Recomendacao: migrar para Qwen3-4B-Instruct-2507 (ja baixado, drop-in). Manter o 35B disponivel apenas para tarefas pontuais de coding agentico que justifiquem ocupar a maquina toda.</t>
         </is>
@@ -2930,7 +3638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C19"/>
+  <dimension ref="B1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2939,176 +3647,224 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="26" t="inlineStr">
+      <c r="B1" s="27" t="inlineStr">
         <is>
           <t>Fontes (coletadas em jun/2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="27" t="inlineStr">
+      <c r="B2" s="28" t="inlineStr">
         <is>
           <t>O que</t>
         </is>
       </c>
-      <c r="C2" s="27" t="inlineStr">
+      <c r="C2" s="28" t="inlineStr">
         <is>
           <t>URL / Referencia</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="28" t="inlineStr">
+      <c r="B3" s="29" t="inlineStr">
         <is>
           <t>Qwen3-4B-Instruct-2507 (benchmarks oficiais)</t>
         </is>
       </c>
-      <c r="C3" s="29" t="inlineStr">
+      <c r="C3" s="30" t="inlineStr">
         <is>
           <t>https://huggingface.co/Qwen/Qwen3-4B-Instruct-2507</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>Qwen3.6-35B-A3B (arquitetura / modelo atual)</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="30" t="inlineStr">
         <is>
           <t>https://qwen.ai/blog?id=qwen3.6-35b-a3b  |  https://huggingface.co/HauhauCS/Qwen3.6-35B-A3B-Uncensored-HauhauCS-Aggressive</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>Qwen3 Technical Report (familia 0.6B-235B)</t>
         </is>
       </c>
-      <c r="C5" s="29" t="inlineStr">
+      <c r="C5" s="30" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2505.09388</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>Qwen3 — guia de specs por tamanho</t>
         </is>
       </c>
-      <c r="C6" s="29" t="inlineStr">
+      <c r="C6" s="30" t="inlineStr">
         <is>
           <t>https://insiderllm.com/guides/qwen3-complete-guide/</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="28" t="inlineStr">
+      <c r="B7" s="29" t="inlineStr">
         <is>
           <t>Gemma 3 (1B/4B/12B/27B)</t>
         </is>
       </c>
-      <c r="C7" s="29" t="inlineStr">
+      <c r="C7" s="30" t="inlineStr">
         <is>
           <t>https://huggingface.co/google/gemma-3-4b-it</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="28" t="inlineStr">
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>Phi-4-mini-instruct (3.8B)</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C8" s="30" t="inlineStr">
         <is>
           <t>https://huggingface.co/microsoft/Phi-4-mini-instruct</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B9" s="29" t="inlineStr">
         <is>
           <t>Llama 3.2 (1B/3B) + Llama 3.1 8B</t>
         </is>
       </c>
-      <c r="C9" s="29" t="inlineStr">
+      <c r="C9" s="30" t="inlineStr">
         <is>
           <t>https://huggingface.co/meta-llama/Llama-3.2-3B-Instruct  |  arXiv:2407.21783</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B10" s="29" t="inlineStr">
         <is>
           <t>Ministral 3 (8B) paper</t>
         </is>
       </c>
-      <c r="C10" s="29" t="inlineStr">
+      <c r="C10" s="30" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2601.08584</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="28" t="inlineStr">
+      <c r="B11" s="29" t="inlineStr">
         <is>
           <t>Llama 3.1 8B — analise comparativa</t>
         </is>
       </c>
-      <c r="C11" s="29" t="inlineStr">
+      <c r="C11" s="30" t="inlineStr">
         <is>
           <t>https://artificialanalysis.ai/models/llama-3-1-instruct-8b</t>
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>Gemma 4 (anuncio oficial)</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>https://blog.google/innovation-and-ai/technology/developers-tools/gemma-4/</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
-      <c r="B13" s="30" t="inlineStr">
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>Gemma 4 (specs E2B/E4B, PLE, function calling, licenca)</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>https://ai.google.dev/gemma/docs/core</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="29" t="inlineStr">
+        <is>
+          <t>MiniMax-M2 GGUF (tamanhos / VRAM minima)</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/unsloth/MiniMax-M2-GGUF</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>MiniMax-M1 (456B, lightning attention) paper</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2506.13585</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="31" t="inlineStr">
         <is>
           <t>Metodologia das colunas de hardware</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="B14" s="31" t="inlineStr">
+    <row r="18" ht="32" customHeight="1">
+      <c r="B18" s="32" t="inlineStr">
         <is>
           <t>GGUF Q4_K_M (GB): tamanho do arquivo no quant Q4_K_M (~4.8 bits/peso). 35B medido = 19.7 GB; demais estimados por params.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="B15" s="31" t="inlineStr">
+    <row r="19" ht="16" customHeight="1">
+      <c r="B19" s="32" t="inlineStr">
         <is>
           <t>Cabe 100% VRAM 8GB?: 'Sim' se modelo+KV+buffers &lt;= ~7 GB (sobra p/ contexto). RX 580 util ~7.4 GB.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="32" customHeight="1">
-      <c r="B16" s="31" t="inlineStr">
+    <row r="20" ht="32" customHeight="1">
+      <c r="B20" s="32" t="inlineStr">
         <is>
           <t>RAM livre est.: de 16 GB, descontando Windows (~3-4 GB) + venv/Whisper/Piper (~2-3 GB). Se o modelo cabe na VRAM, a RAM fica livre.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="32" customHeight="1">
-      <c r="B17" s="31" t="inlineStr">
+    <row r="21" ht="32" customHeight="1">
+      <c r="B21" s="32" t="inlineStr">
         <is>
           <t>Veloc. est. RX580 (tok/s): estimativa memory-bound (RX 580 ~256 GB/s). Modelos na VRAM: rapidos. Com offload p/ CPU: lentos. 35B medido ~5-8 tok/s.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="32" customHeight="1">
-      <c r="B18" s="31" t="inlineStr">
+    <row r="22" ht="32" customHeight="1">
+      <c r="B22" s="32" t="inlineStr">
         <is>
           <t>Benchmarks 'n/d': nao coletados de fonte primaria nesta pesquisa — evitei numeros sem fonte. Colunas Qualidade/PT-BR/Tools sao avaliacao qualitativa do analista.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="32" customHeight="1">
-      <c r="B19" s="31" t="inlineStr">
+    <row r="23" ht="32" customHeight="1">
+      <c r="B23" s="32" t="inlineStr">
         <is>
           <t>Benchmarks nao sao 100% comparaveis entre familias (setups/harness diferentes; thinking vs non-thinking). Use como ordem de grandeza.</t>
         </is>
@@ -3116,11 +3872,11 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B21:C21"/>
     <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B22:C22"/>
     <mergeCell ref="B18:C18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>